<commit_message>
Batch 2: FAST builder, three new labs, faded worked examples, common-mistake feedback
- Module 4: build a FAST diagram yourself (torch part-built, stapler from scratch),
  drag or tap to place, every link checked HOW and WHY, more than one layout accepted
- New labs: function-cost matrix (m3), monthly funnel review (m8), target-cost
  waterfall from shop price to function targets (m13)
- Worked examples that fade into problems for should-cost (m9) and target cost (m13),
  with carry-forward marking and specific feedback for known slips
- Ten common VE mistakes explained when a wrong answer shows one, in the quick checks,
  challenges, practice exam and labs
- Savings Funnel Tracker spreadsheet stages now match Module 8
- New practice test suite

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013T5QQURJq6sk2npuXPPgBh
</commit_message>
<xml_diff>
--- a/toolkit/savings-funnel-tracker.xlsx
+++ b/toolkit/savings-funnel-tracker.xlsx
@@ -557,9 +557,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr"/>
-    </row>
+    <row r="4"/>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
@@ -580,7 +578,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Logged with an owner and a rough saving — no validation yet.</t>
+          <t>Captured with the function, a rough saving and an owner. Nothing checked yet.</t>
         </is>
       </c>
     </row>
@@ -592,31 +590,31 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Business case drafted: saving, one-time cost, risk and validation plan agreed.</t>
+          <t>Technical feasibility confirmed, saving checked by finance, one-time cost estimated.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>L3 · Implemented</t>
+          <t>L3 · Approved</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Change made in production / PPAP cleared.</t>
+          <t>Business case approved by the value board; budget and people committed.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>L4 · Audited</t>
+          <t>L4 · Implemented</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Saving confirmed against the frozen baseline by finance — now it counts.</t>
+          <t>Change in production (PPAP / validation complete) and the saving checked by finance against the fixed starting cost. Only now does it count.</t>
         </is>
       </c>
     </row>
@@ -679,9 +677,8 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr"/>
-    </row>
+    <row r="4"/>
+    <row r="5"/>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
@@ -780,7 +777,7 @@
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>L3 Implemented</t>
+          <t>L3 Approved</t>
         </is>
       </c>
       <c r="D8" s="9" t="n">
@@ -1450,6 +1447,7 @@
         <v/>
       </c>
     </row>
+    <row r="55"/>
     <row r="56" ht="28" customHeight="1">
       <c r="A56" s="14" t="inlineStr">
         <is>
@@ -1457,6 +1455,7 @@
         </is>
       </c>
     </row>
+    <row r="57"/>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
         <is>
@@ -1474,7 +1473,7 @@
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 C21 C22 C23 C24 C25 C26 C27 C28 C29 C30 C31 C32 C33 C34 C35 C36 C37 C38 C39 C40 C41 C42 C43 C44 C45 C46 C47 C48 C49 C50 C51 C52 C53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"L1 Idea,L2 Validated,L3 Implemented,L4 Audited"</formula1>
+      <formula1>"L1 Idea,L2 Validated,L3 Approved,L4 Implemented"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>